<commit_message>
Added sematic layer for japanese character.
</commit_message>
<xml_diff>
--- a/input/ADAS_Scenarios_JP.xlsx
+++ b/input/ADAS_Scenarios_JP.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RAG_11\Language_translation\project\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RAG_11\BASIC_RAG\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FD44660-E11A-4F9C-9B04-B07845D8112A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25DE10B2-7F1D-4B69-BA43-E9769AD2F876}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10276" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="概要 Overview" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="160">
   <si>
     <t>ADAS テストシナリオ仕様書　POC</t>
   </si>
@@ -501,6 +501,9 @@
   </si>
   <si>
     <t>5回</t>
+  </si>
+  <si>
+    <t>車速</t>
   </si>
 </sst>
 </file>
@@ -614,7 +617,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -643,6 +646,15 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -656,16 +668,6 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -980,24 +982,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
     </row>
     <row r="2" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
     </row>
     <row r="4" spans="1:6" ht="26" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
@@ -1117,29 +1119,29 @@
     <col min="2" max="2" width="24" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>
-    <col min="5" max="5" width="14" style="18" customWidth="1"/>
-    <col min="6" max="6" width="60" style="18" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="60" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
     </row>
     <row r="2" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
     </row>
     <row r="3" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="6" t="s">
@@ -1154,8 +1156,8 @@
       <c r="D3" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
     </row>
     <row r="4" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="7" t="s">
@@ -1170,8 +1172,8 @@
       <c r="D4" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="E4" s="16"/>
-      <c r="F4" s="17"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="12"/>
     </row>
     <row r="5" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="4"/>
@@ -1182,8 +1184,8 @@
         <v>35</v>
       </c>
       <c r="D5" s="5"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="17"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="12"/>
     </row>
     <row r="6" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="2"/>
@@ -1194,8 +1196,8 @@
         <v>37</v>
       </c>
       <c r="D6" s="3"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="17"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="12"/>
     </row>
     <row r="7" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="4"/>
@@ -1206,8 +1208,8 @@
         <v>39</v>
       </c>
       <c r="D7" s="5"/>
-      <c r="E7" s="16"/>
-      <c r="F7" s="17"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="12"/>
     </row>
     <row r="8" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="2"/>
@@ -1218,8 +1220,8 @@
         <v>41</v>
       </c>
       <c r="D8" s="3"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="17"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="12"/>
     </row>
     <row r="9" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="4"/>
@@ -1230,8 +1232,8 @@
         <v>41</v>
       </c>
       <c r="D9" s="5"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="17"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="12"/>
     </row>
     <row r="10" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="2"/>
@@ -1242,8 +1244,8 @@
         <v>44</v>
       </c>
       <c r="D10" s="3"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="17"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="12"/>
     </row>
     <row r="11" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="4"/>
@@ -1254,8 +1256,8 @@
         <v>46</v>
       </c>
       <c r="D11" s="5"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="17"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="12"/>
     </row>
     <row r="12" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="2"/>
@@ -1266,8 +1268,8 @@
         <v>48</v>
       </c>
       <c r="D12" s="3"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="17"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="12"/>
     </row>
     <row r="13" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="4"/>
@@ -1278,15 +1280,15 @@
         <v>50</v>
       </c>
       <c r="D13" s="5"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="17"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="12"/>
     </row>
     <row r="15" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="7" t="s">
         <v>51</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>31</v>
+        <v>159</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>32</v>
@@ -1294,8 +1296,8 @@
       <c r="D15" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="E15" s="16"/>
-      <c r="F15" s="17"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="12"/>
     </row>
     <row r="16" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="4"/>
@@ -1306,8 +1308,8 @@
         <v>53</v>
       </c>
       <c r="D16" s="5"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="17"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="12"/>
     </row>
     <row r="17" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="2"/>
@@ -1318,8 +1320,8 @@
         <v>55</v>
       </c>
       <c r="D17" s="3"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="17"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="12"/>
     </row>
     <row r="18" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="4"/>
@@ -1330,8 +1332,8 @@
         <v>37</v>
       </c>
       <c r="D18" s="5"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="17"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="12"/>
     </row>
     <row r="19" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="2"/>
@@ -1342,8 +1344,8 @@
         <v>39</v>
       </c>
       <c r="D19" s="3"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="17"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="12"/>
     </row>
     <row r="20" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="4"/>
@@ -1354,8 +1356,8 @@
         <v>41</v>
       </c>
       <c r="D20" s="5"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="17"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="12"/>
     </row>
     <row r="21" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="2"/>
@@ -1366,8 +1368,8 @@
         <v>41</v>
       </c>
       <c r="D21" s="3"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="17"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="12"/>
     </row>
     <row r="22" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="4"/>
@@ -1378,8 +1380,8 @@
         <v>44</v>
       </c>
       <c r="D22" s="5"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="17"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="12"/>
     </row>
     <row r="23" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="2"/>
@@ -1390,8 +1392,8 @@
         <v>56</v>
       </c>
       <c r="D23" s="3"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="17"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="12"/>
     </row>
     <row r="24" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="4"/>
@@ -1402,8 +1404,8 @@
         <v>46</v>
       </c>
       <c r="D24" s="5"/>
-      <c r="E24" s="16"/>
-      <c r="F24" s="17"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="12"/>
     </row>
     <row r="25" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" s="2"/>
@@ -1414,8 +1416,8 @@
         <v>48</v>
       </c>
       <c r="D25" s="3"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="17"/>
+      <c r="E25" s="11"/>
+      <c r="F25" s="12"/>
     </row>
     <row r="27" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="7" t="s">
@@ -1430,8 +1432,8 @@
       <c r="D27" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="E27" s="16"/>
-      <c r="F27" s="17"/>
+      <c r="E27" s="11"/>
+      <c r="F27" s="12"/>
     </row>
     <row r="28" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="4"/>
@@ -1442,8 +1444,8 @@
         <v>35</v>
       </c>
       <c r="D28" s="5"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="17"/>
+      <c r="E28" s="11"/>
+      <c r="F28" s="12"/>
     </row>
     <row r="29" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="2"/>
@@ -1454,8 +1456,8 @@
         <v>61</v>
       </c>
       <c r="D29" s="3"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="17"/>
+      <c r="E29" s="11"/>
+      <c r="F29" s="12"/>
     </row>
     <row r="30" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="4"/>
@@ -1466,8 +1468,8 @@
         <v>63</v>
       </c>
       <c r="D30" s="5"/>
-      <c r="E30" s="16"/>
-      <c r="F30" s="17"/>
+      <c r="E30" s="11"/>
+      <c r="F30" s="12"/>
     </row>
     <row r="31" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="2"/>
@@ -1478,8 +1480,8 @@
         <v>41</v>
       </c>
       <c r="D31" s="3"/>
-      <c r="E31" s="16"/>
-      <c r="F31" s="17"/>
+      <c r="E31" s="11"/>
+      <c r="F31" s="12"/>
     </row>
     <row r="32" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32" s="4"/>
@@ -1490,8 +1492,8 @@
         <v>41</v>
       </c>
       <c r="D32" s="5"/>
-      <c r="E32" s="16"/>
-      <c r="F32" s="17"/>
+      <c r="E32" s="11"/>
+      <c r="F32" s="12"/>
     </row>
     <row r="33" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" s="2"/>
@@ -1502,8 +1504,8 @@
         <v>44</v>
       </c>
       <c r="D33" s="3"/>
-      <c r="E33" s="16"/>
-      <c r="F33" s="17"/>
+      <c r="E33" s="11"/>
+      <c r="F33" s="12"/>
     </row>
     <row r="34" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="4"/>
@@ -1514,8 +1516,8 @@
         <v>41</v>
       </c>
       <c r="D34" s="5"/>
-      <c r="E34" s="16"/>
-      <c r="F34" s="17"/>
+      <c r="E34" s="11"/>
+      <c r="F34" s="12"/>
     </row>
     <row r="35" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="2"/>
@@ -1526,8 +1528,8 @@
         <v>65</v>
       </c>
       <c r="D35" s="3"/>
-      <c r="E35" s="16"/>
-      <c r="F35" s="17"/>
+      <c r="E35" s="11"/>
+      <c r="F35" s="12"/>
     </row>
     <row r="36" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A36" s="4"/>
@@ -1538,8 +1540,8 @@
         <v>66</v>
       </c>
       <c r="D36" s="5"/>
-      <c r="E36" s="16"/>
-      <c r="F36" s="17"/>
+      <c r="E36" s="11"/>
+      <c r="F36" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1559,29 +1561,29 @@
     <col min="2" max="2" width="24" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>
-    <col min="5" max="5" width="14" style="18" customWidth="1"/>
-    <col min="6" max="6" width="60" style="18" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="60" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
     </row>
     <row r="2" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
     </row>
     <row r="3" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="6" t="s">
@@ -1596,8 +1598,8 @@
       <c r="D3" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
     </row>
     <row r="4" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="7" t="s">
@@ -1612,8 +1614,8 @@
       <c r="D4" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="E4" s="16"/>
-      <c r="F4" s="17"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="12"/>
     </row>
     <row r="5" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="4"/>
@@ -1624,8 +1626,8 @@
         <v>72</v>
       </c>
       <c r="D5" s="5"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="17"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="12"/>
     </row>
     <row r="6" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="2"/>
@@ -1636,8 +1638,8 @@
         <v>74</v>
       </c>
       <c r="D6" s="3"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="17"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="12"/>
     </row>
     <row r="7" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="4"/>
@@ -1648,8 +1650,8 @@
         <v>41</v>
       </c>
       <c r="D7" s="5"/>
-      <c r="E7" s="16"/>
-      <c r="F7" s="17"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="12"/>
     </row>
     <row r="8" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="2"/>
@@ -1660,8 +1662,8 @@
         <v>41</v>
       </c>
       <c r="D8" s="3"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="17"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="12"/>
     </row>
     <row r="9" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="4"/>
@@ -1672,8 +1674,8 @@
         <v>44</v>
       </c>
       <c r="D9" s="5"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="17"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="12"/>
     </row>
     <row r="10" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="2"/>
@@ -1684,8 +1686,8 @@
         <v>44</v>
       </c>
       <c r="D10" s="3"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="17"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="12"/>
     </row>
     <row r="11" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="4"/>
@@ -1696,8 +1698,8 @@
         <v>80</v>
       </c>
       <c r="D11" s="5"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="17"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="12"/>
     </row>
     <row r="12" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="2"/>
@@ -1708,8 +1710,8 @@
         <v>81</v>
       </c>
       <c r="D12" s="3"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="17"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="12"/>
     </row>
     <row r="13" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="4"/>
@@ -1720,8 +1722,8 @@
         <v>82</v>
       </c>
       <c r="D13" s="5"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="17"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="12"/>
     </row>
     <row r="15" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="7" t="s">
@@ -1736,8 +1738,8 @@
       <c r="D15" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="E15" s="16"/>
-      <c r="F15" s="17"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="12"/>
     </row>
     <row r="16" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="4"/>
@@ -1748,8 +1750,8 @@
         <v>86</v>
       </c>
       <c r="D16" s="5"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="17"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="12"/>
     </row>
     <row r="17" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="2"/>
@@ -1760,8 +1762,8 @@
         <v>88</v>
       </c>
       <c r="D17" s="3"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="17"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="12"/>
     </row>
     <row r="18" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="4"/>
@@ -1772,8 +1774,8 @@
         <v>41</v>
       </c>
       <c r="D18" s="5"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="17"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="12"/>
     </row>
     <row r="19" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="2"/>
@@ -1784,8 +1786,8 @@
         <v>41</v>
       </c>
       <c r="D19" s="3"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="17"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="12"/>
     </row>
     <row r="20" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="4"/>
@@ -1796,8 +1798,8 @@
         <v>41</v>
       </c>
       <c r="D20" s="5"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="17"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="12"/>
     </row>
     <row r="21" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="2"/>
@@ -1808,8 +1810,8 @@
         <v>89</v>
       </c>
       <c r="D21" s="3"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="17"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="12"/>
     </row>
     <row r="22" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="4"/>
@@ -1820,8 +1822,8 @@
         <v>91</v>
       </c>
       <c r="D22" s="5"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="17"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="12"/>
     </row>
     <row r="23" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="2"/>
@@ -1832,8 +1834,8 @@
         <v>81</v>
       </c>
       <c r="D23" s="3"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="17"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="12"/>
     </row>
     <row r="24" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="4"/>
@@ -1844,8 +1846,8 @@
         <v>82</v>
       </c>
       <c r="D24" s="5"/>
-      <c r="E24" s="16"/>
-      <c r="F24" s="17"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="12"/>
     </row>
     <row r="26" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="7" t="s">
@@ -1860,8 +1862,8 @@
       <c r="D26" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="E26" s="16"/>
-      <c r="F26" s="17"/>
+      <c r="E26" s="11"/>
+      <c r="F26" s="12"/>
     </row>
     <row r="27" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="4"/>
@@ -1872,8 +1874,8 @@
         <v>95</v>
       </c>
       <c r="D27" s="5"/>
-      <c r="E27" s="16"/>
-      <c r="F27" s="17"/>
+      <c r="E27" s="11"/>
+      <c r="F27" s="12"/>
     </row>
     <row r="28" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="2"/>
@@ -1884,8 +1886,8 @@
         <v>97</v>
       </c>
       <c r="D28" s="3"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="17"/>
+      <c r="E28" s="11"/>
+      <c r="F28" s="12"/>
     </row>
     <row r="29" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="4"/>
@@ -1896,8 +1898,8 @@
         <v>41</v>
       </c>
       <c r="D29" s="5"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="17"/>
+      <c r="E29" s="11"/>
+      <c r="F29" s="12"/>
     </row>
     <row r="30" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="2"/>
@@ -1908,8 +1910,8 @@
         <v>41</v>
       </c>
       <c r="D30" s="3"/>
-      <c r="E30" s="16"/>
-      <c r="F30" s="17"/>
+      <c r="E30" s="11"/>
+      <c r="F30" s="12"/>
     </row>
     <row r="31" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="4"/>
@@ -1920,8 +1922,8 @@
         <v>98</v>
       </c>
       <c r="D31" s="5"/>
-      <c r="E31" s="16"/>
-      <c r="F31" s="17"/>
+      <c r="E31" s="11"/>
+      <c r="F31" s="12"/>
     </row>
     <row r="32" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32" s="2"/>
@@ -1932,8 +1934,8 @@
         <v>100</v>
       </c>
       <c r="D32" s="3"/>
-      <c r="E32" s="16"/>
-      <c r="F32" s="17"/>
+      <c r="E32" s="11"/>
+      <c r="F32" s="12"/>
     </row>
     <row r="33" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" s="4"/>
@@ -1944,8 +1946,8 @@
         <v>101</v>
       </c>
       <c r="D33" s="5"/>
-      <c r="E33" s="16"/>
-      <c r="F33" s="17"/>
+      <c r="E33" s="11"/>
+      <c r="F33" s="12"/>
     </row>
     <row r="34" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="2"/>
@@ -1956,8 +1958,8 @@
         <v>65</v>
       </c>
       <c r="D34" s="3"/>
-      <c r="E34" s="16"/>
-      <c r="F34" s="17"/>
+      <c r="E34" s="11"/>
+      <c r="F34" s="12"/>
     </row>
     <row r="35" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="4"/>
@@ -1968,8 +1970,8 @@
         <v>66</v>
       </c>
       <c r="D35" s="5"/>
-      <c r="E35" s="16"/>
-      <c r="F35" s="17"/>
+      <c r="E35" s="11"/>
+      <c r="F35" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1989,29 +1991,29 @@
     <col min="2" max="2" width="24" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>
-    <col min="5" max="5" width="14" style="18" customWidth="1"/>
-    <col min="6" max="6" width="60" style="18" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="60" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
     </row>
     <row r="2" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
     </row>
     <row r="3" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="6" t="s">
@@ -2026,8 +2028,8 @@
       <c r="D3" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
     </row>
     <row r="4" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="7" t="s">
@@ -2042,8 +2044,8 @@
       <c r="D4" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="E4" s="16"/>
-      <c r="F4" s="17"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="12"/>
     </row>
     <row r="5" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="4"/>
@@ -2054,8 +2056,8 @@
         <v>107</v>
       </c>
       <c r="D5" s="5"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="17"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="12"/>
     </row>
     <row r="6" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="2"/>
@@ -2066,8 +2068,8 @@
         <v>109</v>
       </c>
       <c r="D6" s="3"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="17"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="12"/>
     </row>
     <row r="7" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="4"/>
@@ -2078,8 +2080,8 @@
         <v>111</v>
       </c>
       <c r="D7" s="5"/>
-      <c r="E7" s="16"/>
-      <c r="F7" s="17"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="12"/>
     </row>
     <row r="8" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="2"/>
@@ -2090,8 +2092,8 @@
         <v>113</v>
       </c>
       <c r="D8" s="3"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="17"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="12"/>
     </row>
     <row r="9" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="4"/>
@@ -2102,8 +2104,8 @@
         <v>41</v>
       </c>
       <c r="D9" s="5"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="17"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="12"/>
     </row>
     <row r="10" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="2"/>
@@ -2114,8 +2116,8 @@
         <v>41</v>
       </c>
       <c r="D10" s="3"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="17"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="12"/>
     </row>
     <row r="11" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="4"/>
@@ -2126,8 +2128,8 @@
         <v>41</v>
       </c>
       <c r="D11" s="5"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="17"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="12"/>
     </row>
     <row r="12" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="2"/>
@@ -2138,8 +2140,8 @@
         <v>65</v>
       </c>
       <c r="D12" s="3"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="17"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="12"/>
     </row>
     <row r="13" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="4"/>
@@ -2150,8 +2152,8 @@
         <v>66</v>
       </c>
       <c r="D13" s="5"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="17"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="12"/>
     </row>
     <row r="15" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="7" t="s">
@@ -2166,8 +2168,8 @@
       <c r="D15" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="E15" s="16"/>
-      <c r="F15" s="17"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="12"/>
     </row>
     <row r="16" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="4"/>
@@ -2178,8 +2180,8 @@
         <v>117</v>
       </c>
       <c r="D16" s="5"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="17"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="12"/>
     </row>
     <row r="17" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="2"/>
@@ -2190,8 +2192,8 @@
         <v>119</v>
       </c>
       <c r="D17" s="3"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="17"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="12"/>
     </row>
     <row r="18" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="4"/>
@@ -2202,8 +2204,8 @@
         <v>35</v>
       </c>
       <c r="D18" s="5"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="17"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="12"/>
     </row>
     <row r="19" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="2"/>
@@ -2214,8 +2216,8 @@
         <v>41</v>
       </c>
       <c r="D19" s="3"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="17"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="12"/>
     </row>
     <row r="20" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="4"/>
@@ -2226,8 +2228,8 @@
         <v>41</v>
       </c>
       <c r="D20" s="5"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="17"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="12"/>
     </row>
     <row r="21" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="2"/>
@@ -2238,8 +2240,8 @@
         <v>41</v>
       </c>
       <c r="D21" s="3"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="17"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="12"/>
     </row>
     <row r="22" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="4"/>
@@ -2250,8 +2252,8 @@
         <v>44</v>
       </c>
       <c r="D22" s="5"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="17"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="12"/>
     </row>
     <row r="23" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="2"/>
@@ -2262,8 +2264,8 @@
         <v>121</v>
       </c>
       <c r="D23" s="3"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="17"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="12"/>
     </row>
     <row r="24" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="4"/>
@@ -2274,8 +2276,8 @@
         <v>122</v>
       </c>
       <c r="D24" s="5"/>
-      <c r="E24" s="16"/>
-      <c r="F24" s="17"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="12"/>
     </row>
     <row r="26" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="7" t="s">
@@ -2290,8 +2292,8 @@
       <c r="D26" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="E26" s="16"/>
-      <c r="F26" s="17"/>
+      <c r="E26" s="11"/>
+      <c r="F26" s="12"/>
     </row>
     <row r="27" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="4"/>
@@ -2302,8 +2304,8 @@
         <v>126</v>
       </c>
       <c r="D27" s="5"/>
-      <c r="E27" s="16"/>
-      <c r="F27" s="17"/>
+      <c r="E27" s="11"/>
+      <c r="F27" s="12"/>
     </row>
     <row r="28" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="2"/>
@@ -2314,8 +2316,8 @@
         <v>39</v>
       </c>
       <c r="D28" s="3"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="17"/>
+      <c r="E28" s="11"/>
+      <c r="F28" s="12"/>
     </row>
     <row r="29" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="4"/>
@@ -2326,8 +2328,8 @@
         <v>129</v>
       </c>
       <c r="D29" s="5"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="17"/>
+      <c r="E29" s="11"/>
+      <c r="F29" s="12"/>
     </row>
     <row r="30" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="2"/>
@@ -2338,8 +2340,8 @@
         <v>41</v>
       </c>
       <c r="D30" s="3"/>
-      <c r="E30" s="16"/>
-      <c r="F30" s="17"/>
+      <c r="E30" s="11"/>
+      <c r="F30" s="12"/>
     </row>
     <row r="31" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="4"/>
@@ -2350,8 +2352,8 @@
         <v>41</v>
       </c>
       <c r="D31" s="5"/>
-      <c r="E31" s="16"/>
-      <c r="F31" s="17"/>
+      <c r="E31" s="11"/>
+      <c r="F31" s="12"/>
     </row>
     <row r="32" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32" s="2"/>
@@ -2362,8 +2364,8 @@
         <v>41</v>
       </c>
       <c r="D32" s="3"/>
-      <c r="E32" s="16"/>
-      <c r="F32" s="17"/>
+      <c r="E32" s="11"/>
+      <c r="F32" s="12"/>
     </row>
     <row r="33" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" s="4"/>
@@ -2374,8 +2376,8 @@
         <v>131</v>
       </c>
       <c r="D33" s="5"/>
-      <c r="E33" s="16"/>
-      <c r="F33" s="17"/>
+      <c r="E33" s="11"/>
+      <c r="F33" s="12"/>
     </row>
     <row r="34" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="2"/>
@@ -2386,8 +2388,8 @@
         <v>65</v>
       </c>
       <c r="D34" s="3"/>
-      <c r="E34" s="16"/>
-      <c r="F34" s="17"/>
+      <c r="E34" s="11"/>
+      <c r="F34" s="12"/>
     </row>
     <row r="35" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="4"/>
@@ -2398,8 +2400,8 @@
         <v>66</v>
       </c>
       <c r="D35" s="5"/>
-      <c r="E35" s="16"/>
-      <c r="F35" s="17"/>
+      <c r="E35" s="11"/>
+      <c r="F35" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2419,29 +2421,29 @@
     <col min="2" max="2" width="24" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>
-    <col min="5" max="5" width="14" style="18" customWidth="1"/>
-    <col min="6" max="6" width="60" style="18" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="60" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="17" t="s">
         <v>132</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
     </row>
     <row r="2" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
     </row>
     <row r="3" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="6" t="s">
@@ -2456,8 +2458,8 @@
       <c r="D3" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
     </row>
     <row r="4" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="7" t="s">
@@ -2472,8 +2474,8 @@
       <c r="D4" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="E4" s="16"/>
-      <c r="F4" s="17"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="12"/>
     </row>
     <row r="5" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="4"/>
@@ -2484,8 +2486,8 @@
         <v>135</v>
       </c>
       <c r="D5" s="5"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="17"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="12"/>
     </row>
     <row r="6" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="2"/>
@@ -2496,8 +2498,8 @@
         <v>138</v>
       </c>
       <c r="D6" s="3"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="17"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="12"/>
     </row>
     <row r="7" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="4"/>
@@ -2508,8 +2510,8 @@
         <v>41</v>
       </c>
       <c r="D7" s="5"/>
-      <c r="E7" s="16"/>
-      <c r="F7" s="17"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="12"/>
     </row>
     <row r="8" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="2"/>
@@ -2520,8 +2522,8 @@
         <v>41</v>
       </c>
       <c r="D8" s="3"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="17"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="12"/>
     </row>
     <row r="9" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="4"/>
@@ -2532,8 +2534,8 @@
         <v>35</v>
       </c>
       <c r="D9" s="5"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="17"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="12"/>
     </row>
     <row r="10" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="2"/>
@@ -2544,8 +2546,8 @@
         <v>50</v>
       </c>
       <c r="D10" s="3"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="17"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="12"/>
     </row>
     <row r="11" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="4"/>
@@ -2556,8 +2558,8 @@
         <v>141</v>
       </c>
       <c r="D11" s="5"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="17"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="12"/>
     </row>
     <row r="12" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="2"/>
@@ -2568,8 +2570,8 @@
         <v>142</v>
       </c>
       <c r="D12" s="3"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="17"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="12"/>
     </row>
     <row r="13" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="4"/>
@@ -2580,8 +2582,8 @@
         <v>143</v>
       </c>
       <c r="D13" s="5"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="17"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="12"/>
     </row>
     <row r="15" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="7" t="s">
@@ -2596,8 +2598,8 @@
       <c r="D15" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="E15" s="16"/>
-      <c r="F15" s="17"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="12"/>
     </row>
     <row r="16" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="4"/>
@@ -2608,8 +2610,8 @@
         <v>69</v>
       </c>
       <c r="D16" s="5"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="17"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="12"/>
     </row>
     <row r="17" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="2"/>
@@ -2620,8 +2622,8 @@
         <v>113</v>
       </c>
       <c r="D17" s="3"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="17"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="12"/>
     </row>
     <row r="18" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="4"/>
@@ -2632,8 +2634,8 @@
         <v>149</v>
       </c>
       <c r="D18" s="5"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="17"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="12"/>
     </row>
     <row r="19" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="2"/>
@@ -2644,8 +2646,8 @@
         <v>41</v>
       </c>
       <c r="D19" s="3"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="17"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="12"/>
     </row>
     <row r="20" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="4"/>
@@ -2656,8 +2658,8 @@
         <v>41</v>
       </c>
       <c r="D20" s="5"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="17"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="12"/>
     </row>
     <row r="21" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="2"/>
@@ -2668,8 +2670,8 @@
         <v>41</v>
       </c>
       <c r="D21" s="3"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="17"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="12"/>
     </row>
     <row r="22" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="4"/>
@@ -2680,8 +2682,8 @@
         <v>151</v>
       </c>
       <c r="D22" s="5"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="17"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="12"/>
     </row>
     <row r="23" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="2"/>
@@ -2692,8 +2694,8 @@
         <v>142</v>
       </c>
       <c r="D23" s="3"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="17"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="12"/>
     </row>
     <row r="24" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="4"/>
@@ -2704,8 +2706,8 @@
         <v>143</v>
       </c>
       <c r="D24" s="5"/>
-      <c r="E24" s="16"/>
-      <c r="F24" s="17"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="12"/>
     </row>
     <row r="26" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="7" t="s">
@@ -2720,8 +2722,8 @@
       <c r="D26" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="E26" s="16"/>
-      <c r="F26" s="17"/>
+      <c r="E26" s="11"/>
+      <c r="F26" s="12"/>
     </row>
     <row r="27" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="4"/>
@@ -2732,8 +2734,8 @@
         <v>154</v>
       </c>
       <c r="D27" s="5"/>
-      <c r="E27" s="16"/>
-      <c r="F27" s="17"/>
+      <c r="E27" s="11"/>
+      <c r="F27" s="12"/>
     </row>
     <row r="28" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="2"/>
@@ -2744,8 +2746,8 @@
         <v>158</v>
       </c>
       <c r="D28" s="3"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="17"/>
+      <c r="E28" s="11"/>
+      <c r="F28" s="12"/>
     </row>
     <row r="29" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="4"/>
@@ -2756,8 +2758,8 @@
         <v>149</v>
       </c>
       <c r="D29" s="5"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="17"/>
+      <c r="E29" s="11"/>
+      <c r="F29" s="12"/>
     </row>
     <row r="30" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="2"/>
@@ -2768,8 +2770,8 @@
         <v>41</v>
       </c>
       <c r="D30" s="3"/>
-      <c r="E30" s="16"/>
-      <c r="F30" s="17"/>
+      <c r="E30" s="11"/>
+      <c r="F30" s="12"/>
     </row>
     <row r="31" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="4"/>
@@ -2780,8 +2782,8 @@
         <v>41</v>
       </c>
       <c r="D31" s="5"/>
-      <c r="E31" s="16"/>
-      <c r="F31" s="17"/>
+      <c r="E31" s="11"/>
+      <c r="F31" s="12"/>
     </row>
     <row r="32" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32" s="2"/>
@@ -2792,8 +2794,8 @@
         <v>44</v>
       </c>
       <c r="D32" s="3"/>
-      <c r="E32" s="16"/>
-      <c r="F32" s="17"/>
+      <c r="E32" s="11"/>
+      <c r="F32" s="12"/>
     </row>
     <row r="33" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" s="4"/>
@@ -2804,8 +2806,8 @@
         <v>35</v>
       </c>
       <c r="D33" s="5"/>
-      <c r="E33" s="16"/>
-      <c r="F33" s="17"/>
+      <c r="E33" s="11"/>
+      <c r="F33" s="12"/>
     </row>
     <row r="34" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="2"/>
@@ -2816,8 +2818,8 @@
         <v>46</v>
       </c>
       <c r="D34" s="3"/>
-      <c r="E34" s="16"/>
-      <c r="F34" s="17"/>
+      <c r="E34" s="11"/>
+      <c r="F34" s="12"/>
     </row>
     <row r="35" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="4"/>
@@ -2828,8 +2830,8 @@
         <v>48</v>
       </c>
       <c r="D35" s="5"/>
-      <c r="E35" s="16"/>
-      <c r="F35" s="17"/>
+      <c r="E35" s="11"/>
+      <c r="F35" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>